<commit_message>
kl-term version 2.3.0 added
</commit_message>
<xml_diff>
--- a/term/CodeSystem-CareSocialCodes.xlsx
+++ b/term/CodeSystem-CareSocialCodes.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="299">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.2.0</t>
+    <t>2.3.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-10-31T13:18:46+01:00</t>
+    <t>2025-08-21T08:46:07+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -177,15 +177,6 @@
     <t>VUM Borgerens ressourcer i forhold til indsatsen</t>
   </si>
   <si>
-    <t>54c4ffea-7caf-4edc-8aa9-ef6e0be26c4c</t>
-  </si>
-  <si>
-    <t>FSIII helhedsvurdering</t>
-  </si>
-  <si>
-    <t>Sagsvurdering, der sammenholder resultaterne af en myndighedsudredning og den øvrige sagsoplysning med henblik på at træffe en afgørelse</t>
-  </si>
-  <si>
     <t>7b41185e-eeb4-437d-8120-5d51bbd27a79</t>
   </si>
   <si>
@@ -543,15 +534,6 @@
     <t>udførelse af terapeutfaglig udredning jævnfør FSIII</t>
   </si>
   <si>
-    <t>e70c66c0-a939-493b-8ea8-5b7e7b48ba1a</t>
-  </si>
-  <si>
-    <t>generelle oplysninger, FSIII</t>
-  </si>
-  <si>
-    <t>indhentning af generelle oplysninger jævnfør FSIII</t>
-  </si>
-  <si>
     <t>10deb210-e7e1-4d56-9531-b9ff2102126e</t>
   </si>
   <si>
@@ -562,6 +544,15 @@
   </si>
   <si>
     <t>Det planlagte indsatsforløb er en social indsats, som defineret af FFB, med tilhørende ydelser, målgruppe og tilbud</t>
+  </si>
+  <si>
+    <t>01302bcb-c7f3-42c4-8ded-68e33da064eb</t>
+  </si>
+  <si>
+    <t>Lettilgængelige tilbud til børn og unge i psykisk mistrivsel</t>
+  </si>
+  <si>
+    <t>Forløbskode for lettilgængelige tilbud til børn og unge i psykisk mistrivsel.</t>
   </si>
   <si>
     <t>4fd6c23a-6ff3-4251-ac37-3ca095027b5b</t>
@@ -896,6 +887,30 @@
   </si>
   <si>
     <t>Borger har behov, men har foretaget et aktivt fravalg pga. den omkostning der er forbundet med transport til det sted indsatsen tilbydes</t>
+  </si>
+  <si>
+    <t>880028ec-5f16-4242-ba53-57a902094d5b</t>
+  </si>
+  <si>
+    <t>Deltagere i kontakt</t>
+  </si>
+  <si>
+    <t>ca228a58-bd0e-4b0e-81ce-3866adc26535</t>
+  </si>
+  <si>
+    <t>Barn/ung deltager</t>
+  </si>
+  <si>
+    <t>Behandler og barn/ung i målgruppen (5-17år) og evt. forældre, værger el.lign. er til stede. Barnet/den unge er genstand for journaloptagelsen.</t>
+  </si>
+  <si>
+    <t>d3578249-10df-4051-851d-3986b1570bee</t>
+  </si>
+  <si>
+    <t>Omsorgsperson uden barn/ung</t>
+  </si>
+  <si>
+    <t>Behandling hvor kun behandler og forældre, værger el.lign. til barn/ung er til stede. Barnet/den unge er genstand for journalen.</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1220,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1294,7 +1309,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s" s="2">
         <v>54</v>
@@ -1303,18 +1318,18 @@
         <v>55</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s" s="2">
         <v>57</v>
-      </c>
-      <c r="C8" t="s" s="2">
-        <v>58</v>
       </c>
       <c r="D8" t="s" s="2">
         <v>58</v>
@@ -1392,7 +1407,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>74</v>
@@ -1406,7 +1421,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>77</v>
@@ -1518,21 +1533,21 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="B24" t="s" s="2">
         <v>105</v>
@@ -1546,7 +1561,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B25" t="s" s="2">
         <v>108</v>
@@ -1644,7 +1659,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s" s="2">
         <v>129</v>
@@ -1653,18 +1668,18 @@
         <v>130</v>
       </c>
       <c r="D32" t="s" s="2">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B33" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="C33" t="s" s="2">
         <v>132</v>
-      </c>
-      <c r="C33" t="s" s="2">
-        <v>133</v>
       </c>
       <c r="D33" t="s" s="2">
         <v>133</v>
@@ -1686,7 +1701,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B35" t="s" s="2">
         <v>137</v>
@@ -1695,18 +1710,18 @@
         <v>138</v>
       </c>
       <c r="D35" t="s" s="2">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B36" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="C36" t="s" s="2">
         <v>140</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>141</v>
       </c>
       <c r="D36" t="s" s="2">
         <v>141</v>
@@ -1779,32 +1794,32 @@
         <v>155</v>
       </c>
       <c r="D41" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B42" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="C42" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="C42" t="s" s="2">
-        <v>158</v>
-      </c>
       <c r="D42" t="s" s="2">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B43" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="C43" t="s" s="2">
         <v>159</v>
-      </c>
-      <c r="C43" t="s" s="2">
-        <v>160</v>
       </c>
       <c r="D43" t="s" s="2">
         <v>160</v>
@@ -1868,7 +1883,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B48" t="s" s="2">
         <v>173</v>
@@ -1877,7 +1892,7 @@
         <v>174</v>
       </c>
       <c r="D48" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49">
@@ -1885,27 +1900,27 @@
         <v>43</v>
       </c>
       <c r="B49" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="C49" t="s" s="2">
+        <v>57</v>
+      </c>
+      <c r="D49" t="s" s="2">
         <v>176</v>
-      </c>
-      <c r="C49" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="D49" t="s" s="2">
-        <v>178</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B50" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="C50" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="D50" t="s" s="2">
         <v>179</v>
-      </c>
-      <c r="C50" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="D50" t="s" s="2">
-        <v>180</v>
       </c>
     </row>
     <row r="51">
@@ -1913,24 +1928,24 @@
         <v>43</v>
       </c>
       <c r="B51" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="C51" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="D51" t="s" s="2">
         <v>181</v>
-      </c>
-      <c r="C51" t="s" s="2">
-        <v>60</v>
-      </c>
-      <c r="D51" t="s" s="2">
-        <v>182</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="B52" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="C52" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="C52" t="s" s="2">
-        <v>69</v>
       </c>
       <c r="D52" t="s" s="2">
         <v>184</v>
@@ -1938,7 +1953,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B53" t="s" s="2">
         <v>185</v>
@@ -1952,27 +1967,27 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="B54" t="s" s="2">
         <v>188</v>
       </c>
       <c r="C54" t="s" s="2">
+        <v>69</v>
+      </c>
+      <c r="D54" t="s" s="2">
         <v>189</v>
-      </c>
-      <c r="D54" t="s" s="2">
-        <v>190</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="B55" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="C55" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="C55" t="s" s="2">
-        <v>72</v>
       </c>
       <c r="D55" t="s" s="2">
         <v>192</v>
@@ -1980,7 +1995,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B56" t="s" s="2">
         <v>193</v>
@@ -1994,7 +2009,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="B57" t="s" s="2">
         <v>196</v>
@@ -2008,7 +2023,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B58" t="s" s="2">
         <v>199</v>
@@ -2036,7 +2051,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B60" t="s" s="2">
         <v>205</v>
@@ -2045,18 +2060,18 @@
         <v>206</v>
       </c>
       <c r="D60" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B61" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="C61" t="s" s="2">
         <v>208</v>
-      </c>
-      <c r="C61" t="s" s="2">
-        <v>209</v>
       </c>
       <c r="D61" t="s" s="2">
         <v>209</v>
@@ -2078,7 +2093,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B63" t="s" s="2">
         <v>213</v>
@@ -2087,18 +2102,18 @@
         <v>214</v>
       </c>
       <c r="D63" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B64" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="C64" t="s" s="2">
         <v>216</v>
-      </c>
-      <c r="C64" t="s" s="2">
-        <v>217</v>
       </c>
       <c r="D64" t="s" s="2">
         <v>217</v>
@@ -2162,7 +2177,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B69" t="s" s="2">
         <v>230</v>
@@ -2176,7 +2191,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B70" t="s" s="2">
         <v>233</v>
@@ -2232,7 +2247,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B74" t="s" s="2">
         <v>245</v>
@@ -2241,18 +2256,18 @@
         <v>246</v>
       </c>
       <c r="D74" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B75" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="C75" t="s" s="2">
         <v>248</v>
-      </c>
-      <c r="C75" t="s" s="2">
-        <v>249</v>
       </c>
       <c r="D75" t="s" s="2">
         <v>249</v>
@@ -2316,7 +2331,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B80" t="s" s="2">
         <v>262</v>
@@ -2330,7 +2345,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B81" t="s" s="2">
         <v>265</v>
@@ -2381,7 +2396,7 @@
         <v>275</v>
       </c>
       <c r="D84" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="85">
@@ -2389,10 +2404,10 @@
         <v>43</v>
       </c>
       <c r="B85" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="C85" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="C85" t="s" s="2">
-        <v>278</v>
       </c>
       <c r="D85" t="s" s="2">
         <v>278</v>
@@ -2400,7 +2415,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="B86" t="s" s="2">
         <v>279</v>
@@ -2414,7 +2429,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B87" t="s" s="2">
         <v>282</v>
@@ -2428,7 +2443,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B88" t="s" s="2">
         <v>285</v>
@@ -2442,7 +2457,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B89" t="s" s="2">
         <v>288</v>
@@ -2456,7 +2471,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="B90" t="s" s="2">
         <v>291</v>
@@ -2465,7 +2480,35 @@
         <v>292</v>
       </c>
       <c r="D90" t="s" s="2">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B91" t="s" s="2">
         <v>293</v>
+      </c>
+      <c r="C91" t="s" s="2">
+        <v>294</v>
+      </c>
+      <c r="D91" t="s" s="2">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="B92" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="C92" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="D92" t="s" s="2">
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>